<commit_message>
Updated NZL model - 2025-09-07 02:43
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3560F2-CE1B-42B9-AA96-E78D0D1B7FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17B292A-C922-4554-A347-8D613E547DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="297">
   <si>
     <t>Unit</t>
   </si>
@@ -970,6 +970,9 @@
   </si>
   <si>
     <t>SysCost_Annual</t>
+  </si>
+  <si>
+    <t>f1d</t>
   </si>
 </sst>
 </file>
@@ -4891,11 +4894,11 @@
       </c>
       <c r="C14" t="str">
         <f t="shared" si="1"/>
-        <v>e 1.5 deg no OS.f3d</v>
+        <v>e 1.5 deg no OS.f1d</v>
       </c>
       <c r="H14" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f3d</v>
+        <v>e 1.5 deg no OS.f1d</v>
       </c>
       <c r="I14" t="str">
         <f t="shared" si="3"/>
@@ -4903,7 +4906,7 @@
       </c>
       <c r="J14" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O14">
         <v>9</v>
@@ -5001,7 +5004,7 @@
         <v>263</v>
       </c>
       <c r="U16" t="s">
-        <v>264</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="2:17">
@@ -5259,11 +5262,11 @@
       </c>
       <c r="C25" t="str">
         <f t="shared" si="1"/>
-        <v>d 1.5 deg OS.f3d</v>
+        <v>d 1.5 deg OS.f1d</v>
       </c>
       <c r="H25" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f3d</v>
+        <v>d 1.5 deg OS.f1d</v>
       </c>
       <c r="I25" t="str">
         <f t="shared" si="3"/>
@@ -5271,7 +5274,7 @@
       </c>
       <c r="J25" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O25">
         <v>20</v>
@@ -5600,11 +5603,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f3d</v>
+        <v>c 2 deg (67%).f1d</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f3d</v>
+        <v>c 2 deg (67%).f1d</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -5612,7 +5615,7 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O36">
         <v>31</v>
@@ -5941,11 +5944,11 @@
       </c>
       <c r="C47" t="str">
         <f t="shared" si="6"/>
-        <v>b 2 deg (50%).f3d</v>
+        <v>b 2 deg (50%).f1d</v>
       </c>
       <c r="H47" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f3d</v>
+        <v>b 2 deg (50%).f1d</v>
       </c>
       <c r="I47" t="str">
         <f t="shared" si="3"/>
@@ -5953,7 +5956,7 @@
       </c>
       <c r="J47" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O47">
         <v>42</v>
@@ -6282,11 +6285,11 @@
       </c>
       <c r="C58" t="str">
         <f t="shared" si="7"/>
-        <v>a 3 deg.f3d</v>
+        <v>a 3 deg.f1d</v>
       </c>
       <c r="H58" t="str">
         <f t="shared" si="8"/>
-        <v>a 3 deg.f3d</v>
+        <v>a 3 deg.f1d</v>
       </c>
       <c r="I58" t="str">
         <f t="shared" si="3"/>
@@ -6294,7 +6297,7 @@
       </c>
       <c r="J58" t="str">
         <f t="shared" si="4"/>
-        <v>f3d</v>
+        <v>f1d</v>
       </c>
       <c r="O58">
         <v>53</v>

</xml_diff>

<commit_message>
Updated NZL model - 2025-09-09 22:38
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NZL/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B17B292A-C922-4554-A347-8D613E547DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC5A96E-17E2-474F-8FC2-5215BD4B5D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -879,9 +879,6 @@
     <t>f3d</t>
   </si>
   <si>
-    <t>~TS_Defs: Snk_attr=SANKEY Grid Flows</t>
-  </si>
-  <si>
     <t>~TS_Defs: Snk_attr=SANKEY whole system</t>
   </si>
   <si>
@@ -973,6 +970,9 @@
   </si>
   <si>
     <t>f1d</t>
+  </si>
+  <si>
+    <t>DeACT TS_Defs: Snk_attr=SANKEY Grid Flows</t>
   </si>
 </sst>
 </file>
@@ -4553,7 +4553,7 @@
         <v>230</v>
       </c>
       <c r="Q6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S6">
         <v>1</v>
@@ -4565,7 +4565,7 @@
         <v>244</v>
       </c>
       <c r="W6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="X6" t="s">
         <v>258</v>
@@ -4602,7 +4602,7 @@
         <v>231</v>
       </c>
       <c r="Q7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S7">
         <v>2</v>
@@ -4614,7 +4614,7 @@
         <v>241</v>
       </c>
       <c r="W7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="X7" t="s">
         <v>257</v>
@@ -4651,7 +4651,7 @@
         <v>232</v>
       </c>
       <c r="Q8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S8">
         <v>3</v>
@@ -4663,7 +4663,7 @@
         <v>242</v>
       </c>
       <c r="W8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="X8" t="s">
         <v>256</v>
@@ -4700,7 +4700,7 @@
         <v>233</v>
       </c>
       <c r="Q9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S9">
         <v>4</v>
@@ -4712,7 +4712,7 @@
         <v>240</v>
       </c>
       <c r="W9" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="X9" t="s">
         <v>255</v>
@@ -4749,7 +4749,7 @@
         <v>234</v>
       </c>
       <c r="Q10" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S10">
         <v>5</v>
@@ -4761,7 +4761,7 @@
         <v>247</v>
       </c>
       <c r="W10" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="X10" t="s">
         <v>259</v>
@@ -4795,7 +4795,7 @@
         <v>235</v>
       </c>
       <c r="Q11" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S11">
         <v>6</v>
@@ -4835,7 +4835,7 @@
         <v>236</v>
       </c>
       <c r="Q12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S12">
         <v>7</v>
@@ -4875,7 +4875,7 @@
         <v>237</v>
       </c>
       <c r="Q13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S13">
         <v>8</v>
@@ -4915,7 +4915,7 @@
         <v>263</v>
       </c>
       <c r="Q14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S14">
         <v>9</v>
@@ -4955,7 +4955,7 @@
         <v>238</v>
       </c>
       <c r="Q15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S15">
         <v>10</v>
@@ -4995,7 +4995,7 @@
         <v>239</v>
       </c>
       <c r="Q16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="S16">
         <v>11</v>
@@ -5004,7 +5004,7 @@
         <v>263</v>
       </c>
       <c r="U16" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="17" spans="2:17">
@@ -5035,7 +5035,7 @@
         <v>230</v>
       </c>
       <c r="Q17" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="2:17">
@@ -5066,7 +5066,7 @@
         <v>231</v>
       </c>
       <c r="Q18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="2:17">
@@ -5097,7 +5097,7 @@
         <v>232</v>
       </c>
       <c r="Q19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="2:17">
@@ -5128,7 +5128,7 @@
         <v>233</v>
       </c>
       <c r="Q20" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" spans="2:17">
@@ -5159,7 +5159,7 @@
         <v>234</v>
       </c>
       <c r="Q21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="2:17">
@@ -5190,7 +5190,7 @@
         <v>235</v>
       </c>
       <c r="Q22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="2:17">
@@ -5221,7 +5221,7 @@
         <v>236</v>
       </c>
       <c r="Q23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="2:17">
@@ -5252,7 +5252,7 @@
         <v>237</v>
       </c>
       <c r="Q24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="25" spans="2:17">
@@ -5283,7 +5283,7 @@
         <v>263</v>
       </c>
       <c r="Q25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" spans="2:17">
@@ -5314,7 +5314,7 @@
         <v>238</v>
       </c>
       <c r="Q26" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27" spans="2:17">
@@ -5345,7 +5345,7 @@
         <v>239</v>
       </c>
       <c r="Q27" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="28" spans="2:17">
@@ -5376,7 +5376,7 @@
         <v>230</v>
       </c>
       <c r="Q28" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="29" spans="2:17">
@@ -5407,7 +5407,7 @@
         <v>231</v>
       </c>
       <c r="Q29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="2:17">
@@ -5438,7 +5438,7 @@
         <v>232</v>
       </c>
       <c r="Q30" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="31" spans="2:17">
@@ -5469,7 +5469,7 @@
         <v>233</v>
       </c>
       <c r="Q31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="32" spans="2:17">
@@ -5500,7 +5500,7 @@
         <v>234</v>
       </c>
       <c r="Q32" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="33" spans="2:17">
@@ -5531,7 +5531,7 @@
         <v>235</v>
       </c>
       <c r="Q33" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="2:17">
@@ -5562,7 +5562,7 @@
         <v>236</v>
       </c>
       <c r="Q34" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="2:17">
@@ -5593,7 +5593,7 @@
         <v>237</v>
       </c>
       <c r="Q35" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="2:17">
@@ -5624,7 +5624,7 @@
         <v>263</v>
       </c>
       <c r="Q36" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" spans="2:17">
@@ -5655,7 +5655,7 @@
         <v>238</v>
       </c>
       <c r="Q37" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="2:17">
@@ -5686,7 +5686,7 @@
         <v>239</v>
       </c>
       <c r="Q38" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="39" spans="2:17">
@@ -5717,7 +5717,7 @@
         <v>230</v>
       </c>
       <c r="Q39" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="2:17">
@@ -5748,7 +5748,7 @@
         <v>231</v>
       </c>
       <c r="Q40" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="2:17">
@@ -5779,7 +5779,7 @@
         <v>232</v>
       </c>
       <c r="Q41" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="42" spans="2:17">
@@ -5810,7 +5810,7 @@
         <v>233</v>
       </c>
       <c r="Q42" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="43" spans="2:17">
@@ -5841,7 +5841,7 @@
         <v>234</v>
       </c>
       <c r="Q43" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="2:17">
@@ -5872,7 +5872,7 @@
         <v>235</v>
       </c>
       <c r="Q44" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="2:17">
@@ -5903,7 +5903,7 @@
         <v>236</v>
       </c>
       <c r="Q45" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="2:17">
@@ -5934,7 +5934,7 @@
         <v>237</v>
       </c>
       <c r="Q46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="47" spans="2:17">
@@ -5965,7 +5965,7 @@
         <v>263</v>
       </c>
       <c r="Q47" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="48" spans="2:17">
@@ -5996,7 +5996,7 @@
         <v>238</v>
       </c>
       <c r="Q48" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="49" spans="2:17">
@@ -6027,7 +6027,7 @@
         <v>239</v>
       </c>
       <c r="Q49" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="50" spans="2:17">
@@ -6058,7 +6058,7 @@
         <v>230</v>
       </c>
       <c r="Q50" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="51" spans="2:17">
@@ -6089,7 +6089,7 @@
         <v>231</v>
       </c>
       <c r="Q51" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="52" spans="2:17">
@@ -6120,7 +6120,7 @@
         <v>232</v>
       </c>
       <c r="Q52" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="53" spans="2:17">
@@ -6151,7 +6151,7 @@
         <v>233</v>
       </c>
       <c r="Q53" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="2:17">
@@ -6182,7 +6182,7 @@
         <v>234</v>
       </c>
       <c r="Q54" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" spans="2:17">
@@ -6213,7 +6213,7 @@
         <v>235</v>
       </c>
       <c r="Q55" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" spans="2:17">
@@ -6244,7 +6244,7 @@
         <v>236</v>
       </c>
       <c r="Q56" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="57" spans="2:17">
@@ -6275,7 +6275,7 @@
         <v>237</v>
       </c>
       <c r="Q57" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" spans="2:17">
@@ -6306,7 +6306,7 @@
         <v>263</v>
       </c>
       <c r="Q58" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="59" spans="2:17">
@@ -6337,7 +6337,7 @@
         <v>238</v>
       </c>
       <c r="Q59" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="60" spans="2:17">
@@ -6368,7 +6368,7 @@
         <v>239</v>
       </c>
       <c r="Q60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -6605,7 +6605,7 @@
         <v>117</v>
       </c>
       <c r="K9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="N9" t="s">
         <v>82</v>
@@ -6687,13 +6687,13 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K14" t="s">
+        <v>292</v>
+      </c>
+      <c r="N14" t="s">
         <v>293</v>
-      </c>
-      <c r="N14" t="s">
-        <v>294</v>
       </c>
       <c r="Q14" t="s">
         <v>50</v>
@@ -6701,13 +6701,13 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="K15" t="s">
         <v>292</v>
       </c>
-      <c r="K15" t="s">
-        <v>293</v>
-      </c>
       <c r="N15" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q15" t="s">
         <v>50</v>
@@ -6812,7 +6812,7 @@
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -6920,7 +6920,7 @@
     </row>
     <row r="10" spans="1:19" ht="17.25" thickBot="1">
       <c r="A10" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -6987,7 +6987,7 @@
         <v>120</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -7006,7 +7006,7 @@
         <v>160</v>
       </c>
       <c r="M13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S13">
         <v>-1</v>
@@ -7028,7 +7028,7 @@
         <v>160</v>
       </c>
       <c r="M14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="S14">
         <v>-1</v>
@@ -7039,7 +7039,7 @@
         <v>120</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -7058,7 +7058,7 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S16">
         <v>-1</v>
@@ -7080,7 +7080,7 @@
         <v>160</v>
       </c>
       <c r="M17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="S17">
         <v>-1</v>
@@ -7091,7 +7091,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -7109,7 +7109,7 @@
         <v>160</v>
       </c>
       <c r="M19" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S19">
         <v>-1</v>
@@ -7130,7 +7130,7 @@
         <v>160</v>
       </c>
       <c r="M20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="S20">
         <v>-1</v>
@@ -7150,7 +7150,7 @@
         <v>160</v>
       </c>
       <c r="M23" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="S23">
         <v>-1</v>
@@ -7274,7 +7274,7 @@
         <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7282,7 +7282,7 @@
         <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -7815,7 +7815,7 @@
         <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -7823,7 +7823,7 @@
         <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -7840,7 +7840,7 @@
         <v>187</v>
       </c>
       <c r="B27" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -7977,7 +7977,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -7986,7 +7986,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -8013,7 +8013,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -8022,7 +8022,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -8031,18 +8031,18 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>